<commit_message>
County-first template and checks; 22 ASAL counties
</commit_message>
<xml_diff>
--- a/docs/drought_relief_disbursement_template.xlsx
+++ b/docs/drought_relief_disbursement_template.xlsx
@@ -1469,8 +1469,10 @@
       <c r="B15" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>277</v>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Enter the total disbursed in that ward-month as a plain number, with no currency symbol or thousands separator, and choose the currency in the next column: KES or USD. If aid was in kind, enter "not applicable" as the amount and choose "Not applicable (in kind)" as the unit. If an estimated monetary value of the in-kind transfers is available, please add it in Notes.</t>
+        </is>
       </c>
     </row>
     <row r="17" spans="2:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1493,8 +1495,10 @@
       <c r="B21" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="28" t="s">
-        <v>265</v>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All 125 wards in scope are on the 'Lists' tab (columns A-B), with their county. On the Data tab, choose the County first (column A); the Ward drop-down (column B) then shows only that county's wards. Please double check for completeness with the provided list.</t>
+        </is>
       </c>
     </row>
     <row r="22" spans="2:11" ht="70" x14ac:dyDescent="0.2">
@@ -1519,10 +1523,10 @@
     <row r="27" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B28" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="13" t="s">
         <v>15</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>16</v>
       </c>
       <c r="D28" s="13" t="s">
         <v>17</v>
@@ -1551,10 +1555,10 @@
     </row>
     <row r="29" spans="2:11" s="30" customFormat="1" ht="26" x14ac:dyDescent="0.2">
       <c r="B29" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" s="29" t="s">
         <v>24</v>
-      </c>
-      <c r="C29" s="29" t="s">
-        <v>25</v>
       </c>
       <c r="D29" s="29" t="s">
         <v>26</v>
@@ -1583,10 +1587,10 @@
     </row>
     <row r="30" spans="2:11" s="30" customFormat="1" ht="26" x14ac:dyDescent="0.2">
       <c r="B30" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="29" t="s">
         <v>24</v>
-      </c>
-      <c r="C30" s="29" t="s">
-        <v>25</v>
       </c>
       <c r="D30" s="29" t="s">
         <v>26</v>
@@ -1615,10 +1619,10 @@
     </row>
     <row r="31" spans="2:11" s="30" customFormat="1" ht="52" x14ac:dyDescent="0.2">
       <c r="B31" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="29" t="s">
         <v>24</v>
-      </c>
-      <c r="C31" s="29" t="s">
-        <v>25</v>
       </c>
       <c r="D31" s="29" t="s">
         <v>26</v>
@@ -1629,8 +1633,10 @@
       <c r="F31" s="31" t="s">
         <v>278</v>
       </c>
-      <c r="G31" s="29" t="s">
-        <v>278</v>
+      <c r="G31" s="29" t="inlineStr">
+        <is>
+          <t>Not applicable (in kind)</t>
+        </is>
       </c>
       <c r="H31" s="29">
         <v>100</v>
@@ -1673,7 +1679,7 @@
         <v>36</v>
       </c>
       <c r="C36" s="16">
-        <f>SUMPRODUCT((Data!$A$3:$A$1500&lt;&gt;"")/COUNTIF(Data!$A$3:$A$1500,Data!$A$3:$A$1500&amp;""))</f>
+        <f>SUMPRODUCT((Data!$B$3:$B$1500&lt;&gt;"")/COUNTIF(Data!$B$3:$B$1500,Data!$B$3:$B$1500&amp;""))</f>
         <v>0</v>
       </c>
     </row>
@@ -1731,8 +1737,8 @@
   <dimension ref="A1:J1002"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
@@ -1761,10 +1767,10 @@
     </row>
     <row r="2" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>15</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>16</v>
       </c>
       <c r="C2" s="17" t="s">
         <v>17</v>
@@ -13812,23 +13818,23 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
-        <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" errorTitle="Ward not on the requested list" error="This ward is not on the list of 125 wards we circulated. Please double-check the spelling; keep it if it is correct and flag it in the Notes column." xr:uid="{00000000-0002-0000-0100-000000000000}">
+        <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" errorTitle="Ward not on the requested list" error="This ward is not on the list for the county chosen in column A. Choose the county first, then the ward. If the ward is correct, keep it and explain in the Notes column." xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
-            <xm:f>Lists!$A$2:$A$126</xm:f>
+            <xm:f>OFFSET(Lists!$B$1,MATCH($A3,Lists!$A$2:$A$126,0),0,COUNTIF(Lists!$A$2:$A$126,$A3),1)</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>B3:B1002</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" errorStyle="stop" showErrorMessage="1" allowBlank="1" errorTitle="County not on list" error="Choose one of the 22 counties from the drop-down." xr:uid="{00000000-0002-0000-0100-000001000000}">
+          <x14:formula1>
+            <xm:f>Lists!$P$2:$P$23</xm:f>
           </x14:formula1>
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
           <xm:sqref>A3:A1002</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" errorTitle="County not on list" error="Please choose the county from the drop-down." xr:uid="{00000000-0002-0000-0100-000001000000}">
-          <x14:formula1>
-            <xm:f>Lists!$B$2:$B$48</xm:f>
-          </x14:formula1>
-          <x14:formula2>
-            <xm:f>0</xm:f>
-          </x14:formula2>
-          <xm:sqref>B3:B1002</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" errorTitle="Check the month format" error="Please use YYYY-MM, e.g. 2024-03. One month per row — no quarters or ranges." xr:uid="{00000000-0002-0000-0100-000002000000}">
           <x14:formula1>
@@ -13857,9 +13863,9 @@
           </x14:formula2>
           <xm:sqref>I3:I1002</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" errorTitle="Unit not on list" error="Please state the currency or physical unit of the amount." xr:uid="{00000000-0002-0000-0100-000004000000}">
+        <x14:dataValidation type="list" errorStyle="stop" allowBlank="1" showErrorMessage="1" errorTitle="Choose from the list" error="Currency / unit must be KES, USD, or Not applicable (in kind)." xr:uid="{00000000-0002-0000-0100-000004000000}">
           <x14:formula1>
-            <xm:f>Lists!$E$2:$E$20</xm:f>
+            <xm:f>Lists!$E$2:$E$4</xm:f>
           </x14:formula1>
           <x14:formula2>
             <xm:f>0</xm:f>
@@ -13874,18 +13880,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:P126"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="26" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>16</v>
+    <row r="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">County</t>
+        </is>
+      </c>
+      <c r="B1" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ward</t>
+        </is>
       </c>
       <c r="C1" s="23" t="s">
         <v>42</v>
@@ -13899,13 +13910,22 @@
       <c r="F1" s="23" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>46</v>
+      <c r="P1" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">County (drop-down)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" x14ac:dyDescent="0.2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Churo/Amaya</t>
+        </is>
       </c>
       <c r="C2" s="24" t="s">
         <v>47</v>
@@ -13919,13 +13939,22 @@
       <c r="F2" s="24" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>50</v>
+      <c r="P2" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ilchamus</t>
+        </is>
       </c>
       <c r="C3" s="24" t="s">
         <v>51</v>
@@ -13939,13 +13968,22 @@
       <c r="F3" s="24" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>55</v>
+      <c r="P3" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kolowa</t>
+        </is>
       </c>
       <c r="C4" s="24" t="s">
         <v>26</v>
@@ -13953,8 +13991,10 @@
       <c r="D4" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="24" t="s">
-        <v>72</v>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>Not applicable (in kind)</t>
+        </is>
       </c>
       <c r="F4" s="24" t="s">
         <v>57</v>
@@ -13968,13 +14008,22 @@
       <c r="M4" s="25"/>
       <c r="N4" s="25"/>
       <c r="O4" s="25"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>59</v>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mukutani</t>
+        </is>
       </c>
       <c r="C5" s="24" t="s">
         <v>60</v>
@@ -13997,13 +14046,22 @@
       <c r="M5" s="25"/>
       <c r="N5" s="25"/>
       <c r="O5" s="25"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>64</v>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ribikwo</t>
+        </is>
       </c>
       <c r="C6" s="24" t="s">
         <v>65</v>
@@ -14016,8 +14074,10 @@
         <v>67</v>
       </c>
       <c r="G6" s="25"/>
-      <c r="H6" s="27" t="s">
-        <v>44</v>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Columns A-B: the 125 wards in scope and their county, sorted by county. The Ward drop-down on the Data tab shows only the wards of the county chosen in column A. Column P: the 22 counties.</t>
+        </is>
       </c>
       <c r="I6" s="25"/>
       <c r="J6" s="25"/>
@@ -14026,13 +14086,22 @@
       <c r="M6" s="25"/>
       <c r="N6" s="25"/>
       <c r="O6" s="25"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>69</v>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" x14ac:dyDescent="0.2">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saimo/Kipsaraman</t>
+        </is>
       </c>
       <c r="C7" s="24" t="s">
         <v>70</v>
@@ -14052,13 +14121,22 @@
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>75</v>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baringo</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tangulbei/Korossi</t>
+        </is>
       </c>
       <c r="C8" s="24" t="s">
         <v>76</v>
@@ -14069,13 +14147,22 @@
       <c r="F8" s="24" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>80</v>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embu</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evurore</t>
+        </is>
       </c>
       <c r="C9" s="24" t="s">
         <v>81</v>
@@ -14083,13 +14170,22 @@
       <c r="D9" s="24" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>84</v>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kwale</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embu</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kiambere</t>
+        </is>
       </c>
       <c r="C10" s="24" t="s">
         <v>85</v>
@@ -14097,13 +14193,22 @@
       <c r="D10" s="24" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>87</v>
+      <c r="P10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laikipia</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" x14ac:dyDescent="0.2">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abakaile</t>
+        </is>
       </c>
       <c r="C11" s="24" t="s">
         <v>88</v>
@@ -14111,757 +14216,1536 @@
       <c r="D11" s="24" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>91</v>
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lamu</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" x14ac:dyDescent="0.2">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Iftin</t>
+        </is>
       </c>
       <c r="C12" s="24" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>94</v>
+      <c r="P12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" x14ac:dyDescent="0.2">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ijara</t>
+        </is>
       </c>
       <c r="C13" s="24" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>97</v>
+      <c r="P13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandera</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" x14ac:dyDescent="0.2">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liboi</t>
+        </is>
       </c>
       <c r="C14" s="24" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>100</v>
+      <c r="P14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" x14ac:dyDescent="0.2">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maalamin</t>
+        </is>
       </c>
       <c r="C15" s="24" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>103</v>
+      <c r="P15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meru</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nanighi</t>
+        </is>
       </c>
       <c r="C16" s="24" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>106</v>
+      <c r="P16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Narok</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garissa</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saka</t>
+        </is>
       </c>
       <c r="C17" s="24" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>109</v>
+      <c r="P17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nyeri</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" x14ac:dyDescent="0.2">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bulla Pesa</t>
+        </is>
       </c>
       <c r="C18" s="24" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>112</v>
+      <c r="P18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samburu</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" x14ac:dyDescent="0.2">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Burat</t>
+        </is>
       </c>
       <c r="C19" s="24" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>115</v>
+      <c r="P19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taita Taveta</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" x14ac:dyDescent="0.2">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chari</t>
+        </is>
       </c>
       <c r="C20" s="24" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>118</v>
+      <c r="P20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tana River</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" x14ac:dyDescent="0.2">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cherab</t>
+        </is>
       </c>
       <c r="C21" s="24" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>121</v>
+      <c r="P21" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" x14ac:dyDescent="0.2">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kinna</t>
+        </is>
       </c>
       <c r="C22" s="24" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>124</v>
+      <c r="P22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wajir</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" x14ac:dyDescent="0.2">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oldo-nyiro</t>
+        </is>
       </c>
       <c r="C23" s="24" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>127</v>
+      <c r="P23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Pokot</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" x14ac:dyDescent="0.2">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isiolo</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sericho</t>
+        </is>
       </c>
       <c r="C24" s="24" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>130</v>
+    <row r="25" x14ac:dyDescent="0.2">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dalalekutuk</t>
+        </is>
       </c>
       <c r="C25" s="24" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>25</v>
+    <row r="26" x14ac:dyDescent="0.2">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ewuaso O o Nkidong'i/M</t>
+        </is>
       </c>
       <c r="C26" s="24" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="B27" s="10" t="s">
-        <v>135</v>
+    <row r="27" x14ac:dyDescent="0.2">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Iloodokilani</t>
+        </is>
       </c>
       <c r="C27" s="24" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>138</v>
+    <row r="28" x14ac:dyDescent="0.2">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Imbirikani/Eselenkei</t>
+        </is>
       </c>
       <c r="C28" s="24" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>141</v>
+    <row r="29" x14ac:dyDescent="0.2">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kaputei North</t>
+        </is>
       </c>
       <c r="C29" s="24" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>144</v>
+    <row r="30" x14ac:dyDescent="0.2">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magadi</t>
+        </is>
       </c>
       <c r="C30" s="24" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>147</v>
+    <row r="31" x14ac:dyDescent="0.2">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kajiado</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rombo</t>
+        </is>
       </c>
       <c r="C31" s="24" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>150</v>
+    <row r="32" x14ac:dyDescent="0.2">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adu</t>
+        </is>
       </c>
       <c r="C32" s="24" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>153</v>
+    <row r="33" x14ac:dyDescent="0.2">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bamba</t>
+        </is>
       </c>
       <c r="C33" s="24" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="B44" s="10" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="B45" s="10" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" s="10" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" s="10" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" s="10" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" s="10" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" s="10" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A54" s="10" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A55" s="10" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A56" s="10" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A57" s="10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A58" s="10" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A59" s="10" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A60" s="10" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A61" s="10" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A62" s="10" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A63" s="10" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A64" s="10" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A65" s="10" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A66" s="10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A67" s="10" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A68" s="10" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A69" s="10" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A70" s="10" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A71" s="10" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A72" s="10" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A73" s="10" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A74" s="10" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A75" s="10" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A76" s="10" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A77" s="10" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A78" s="10" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A79" s="10" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A80" s="10" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A81" s="10" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A82" s="10" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A83" s="10" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A84" s="10" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A85" s="10" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A86" s="10" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A87" s="10" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A88" s="10" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A89" s="10" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A90" s="10" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A91" s="10" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A92" s="10" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A93" s="10" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A94" s="10" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A95" s="10" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A96" s="10" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A97" s="10" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A98" s="10" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A99" s="10" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" s="10" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A101" s="10" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A102" s="10" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A103" s="10" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A104" s="10" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A105" s="10" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A106" s="10" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A107" s="10" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A108" s="10" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A109" s="10" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A110" s="10" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A111" s="10" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A112" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A113" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A114" s="10" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A115" s="10" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A116" s="10" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A117" s="10" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A118" s="10" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A119" s="10" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A120" s="10" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A121" s="10" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A122" s="10" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A123" s="10" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A124" s="10" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A125" s="10" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A126" s="10" t="s">
-        <v>261</v>
+    <row r="34" x14ac:dyDescent="0.2">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jaribuni</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" x14ac:dyDescent="0.2">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kakuyuni</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" x14ac:dyDescent="0.2">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mwanamwinga</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" x14ac:dyDescent="0.2">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mwarakaya</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" x14ac:dyDescent="0.2">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilifi</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mwawesa</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" x14ac:dyDescent="0.2">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikutha</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" x14ac:dyDescent="0.2">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kanyangi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" x14ac:dyDescent="0.2">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kauwi</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" x14ac:dyDescent="0.2">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kivou</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" x14ac:dyDescent="0.2">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Malalani/Endau</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" x14ac:dyDescent="0.2">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migwani</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" x14ac:dyDescent="0.2">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nuu</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" x14ac:dyDescent="0.2">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitui</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tseikuru</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" x14ac:dyDescent="0.2">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kwale</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kasemani</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" x14ac:dyDescent="0.2">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kwale</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mwereni</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" x14ac:dyDescent="0.2">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kwale</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ndavaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" x14ac:dyDescent="0.2">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kwale</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Waa</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" x14ac:dyDescent="0.2">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laikipia</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mukogodo East</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" x14ac:dyDescent="0.2">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laikipia</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mukogodo West</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" x14ac:dyDescent="0.2">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laikipia</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngobit</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" x14ac:dyDescent="0.2">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laikipia</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sosiani</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" x14ac:dyDescent="0.2">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lamu</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bahari</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" x14ac:dyDescent="0.2">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lamu</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faza</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" x14ac:dyDescent="0.2">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lamu</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kiunga</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" x14ac:dyDescent="0.2">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lamu</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Witu</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" x14ac:dyDescent="0.2">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kasikeu/Kiou</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" x14ac:dyDescent="0.2">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kithungo/Kitundu</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" x14ac:dyDescent="0.2">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitise/Kithuki</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" x14ac:dyDescent="0.2">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Masongaleni</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" x14ac:dyDescent="0.2">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Masumba/Nguu</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" x14ac:dyDescent="0.2">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mukaa</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" x14ac:dyDescent="0.2">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Makueni</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ukia</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" x14ac:dyDescent="0.2">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandera</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dandu</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" x14ac:dyDescent="0.2">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandera</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kalaliyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" x14ac:dyDescent="0.2">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandera</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kutulo</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" x14ac:dyDescent="0.2">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandera</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rhamu Dimtu</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" x14ac:dyDescent="0.2">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandera</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shimbir Fatuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" x14ac:dyDescent="0.2">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandera</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Waranqara</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" x14ac:dyDescent="0.2">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Butiye</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" x14ac:dyDescent="0.2">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Golbo</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" x14ac:dyDescent="0.2">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karare</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" x14ac:dyDescent="0.2">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Korr/Ngurunit</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" x14ac:dyDescent="0.2">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loiyangalani</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" x14ac:dyDescent="0.2">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Merigi</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" x14ac:dyDescent="0.2">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sagante/Jaldessa</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" x14ac:dyDescent="0.2">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turbi</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" x14ac:dyDescent="0.2">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marsabit</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uran</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" x14ac:dyDescent="0.2">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meru</t>
+        </is>
+      </c>
+      <c r="B81" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Akithi</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" x14ac:dyDescent="0.2">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meru</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kangeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" x14ac:dyDescent="0.2">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meru</t>
+        </is>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mikinduri</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" x14ac:dyDescent="0.2">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Narok</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ilkerin</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" x14ac:dyDescent="0.2">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Narok</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilgoris Central</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" x14ac:dyDescent="0.2">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Narok</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maji Moto/Naroosura</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" x14ac:dyDescent="0.2">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Narok</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mosiro (Narok East)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" x14ac:dyDescent="0.2">
+      <c r="A88" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Narok</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nkareta</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" x14ac:dyDescent="0.2">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Narok</t>
+        </is>
+      </c>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Siana</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" x14ac:dyDescent="0.2">
+      <c r="A90" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nyeri</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mugunda</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" x14ac:dyDescent="0.2">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nyeri</t>
+        </is>
+      </c>
+      <c r="B91" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thegu River</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" x14ac:dyDescent="0.2">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samburu</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nachola</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" x14ac:dyDescent="0.2">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samburu</t>
+        </is>
+      </c>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ndoto</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" x14ac:dyDescent="0.2">
+      <c r="A94" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samburu</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suguta Marmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" x14ac:dyDescent="0.2">
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samburu</t>
+        </is>
+      </c>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wamba North</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" x14ac:dyDescent="0.2">
+      <c r="A96" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samburu</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wamba West</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" x14ac:dyDescent="0.2">
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samburu</t>
+        </is>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Waso</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" x14ac:dyDescent="0.2">
+      <c r="A98" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taita Taveta</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chala</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" x14ac:dyDescent="0.2">
+      <c r="A99" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taita Taveta</t>
+        </is>
+      </c>
+      <c r="B99" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kasigau</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" x14ac:dyDescent="0.2">
+      <c r="A100" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taita Taveta</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mboghoni</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" x14ac:dyDescent="0.2">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taita Taveta</t>
+        </is>
+      </c>
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngolia</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" x14ac:dyDescent="0.2">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tana River</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bangale</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" x14ac:dyDescent="0.2">
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tana River</t>
+        </is>
+      </c>
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chewani</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" x14ac:dyDescent="0.2">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tana River</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Garsen Central</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" x14ac:dyDescent="0.2">
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tana River</t>
+        </is>
+      </c>
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kipini East</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" x14ac:dyDescent="0.2">
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tana River</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Madogo</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" x14ac:dyDescent="0.2">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tana River</t>
+        </is>
+      </c>
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wayu</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" x14ac:dyDescent="0.2">
+      <c r="A108" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+      <c r="B108" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kaeris</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" x14ac:dyDescent="0.2">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kakuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" x14ac:dyDescent="0.2">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kapedo/Napeitom</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" x14ac:dyDescent="0.2">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Katilu</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" x14ac:dyDescent="0.2">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lake Zone</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" x14ac:dyDescent="0.2">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lokichar</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" x14ac:dyDescent="0.2">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkana</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turkwel</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" x14ac:dyDescent="0.2">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wajir</t>
+        </is>
+      </c>
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Barwago</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" x14ac:dyDescent="0.2">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wajir</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bute</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" x14ac:dyDescent="0.2">
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wajir</t>
+        </is>
+      </c>
+      <c r="B117" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dela</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" x14ac:dyDescent="0.2">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wajir</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hadado/Adhibohol</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" x14ac:dyDescent="0.2">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wajir</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lagboghol South</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" x14ac:dyDescent="0.2">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wajir</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarbaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" x14ac:dyDescent="0.2">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Pokot</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chepareria</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" x14ac:dyDescent="0.2">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Pokot</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kapchoki</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" x14ac:dyDescent="0.2">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Pokot</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kapenguria</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" x14ac:dyDescent="0.2">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Pokot</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Masol</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" x14ac:dyDescent="0.2">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Pokot</t>
+        </is>
+      </c>
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Riwo</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" x14ac:dyDescent="0.2">
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West Pokot</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wei Wei</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>